<commit_message>
delivery v3.8: OCBS=6 items, CWBS=5 items per project spec
</commit_message>
<xml_diff>
--- a/results/主模型结果填答表.xlsx
+++ b/results/主模型结果填答表.xlsx
@@ -1966,10 +1966,10 @@
         </is>
       </c>
       <c r="B3" s="15" t="n">
-        <v>30.712</v>
+        <v>30.773</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>4.72</v>
+        <v>4.638</v>
       </c>
       <c r="D3" s="15" t="inlineStr"/>
       <c r="E3" s="15" t="n">
@@ -1999,14 +1999,14 @@
         </is>
       </c>
       <c r="B4" s="15" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="C4" s="15" t="n">
         <v>0.497</v>
       </c>
       <c r="D4" s="15" t="inlineStr"/>
       <c r="E4" s="15" t="n">
-        <v>0.029</v>
+        <v>0.024</v>
       </c>
       <c r="F4" s="15" t="n">
         <v>1</v>
@@ -2034,17 +2034,17 @@
         </is>
       </c>
       <c r="B5" s="15" t="n">
-        <v>3.079</v>
+        <v>3.104</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="D5" s="15" t="inlineStr"/>
       <c r="E5" s="15" t="n">
-        <v>-0</v>
+        <v>-0.005</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>-0.046</v>
+        <v>-0.054</v>
       </c>
       <c r="G5" s="15" t="n">
         <v>1</v>
@@ -2071,20 +2071,20 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>2.555</v>
+        <v>2.577</v>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1.132</v>
+        <v>1.145</v>
       </c>
       <c r="D6" s="15" t="inlineStr"/>
       <c r="E6" s="15" t="n">
-        <v>-0.045</v>
+        <v>-0.038</v>
       </c>
       <c r="F6" s="15" t="n">
-        <v>-0.034</v>
+        <v>-0.041</v>
       </c>
       <c r="G6" s="15" t="n">
-        <v>-0.017</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>1</v>
@@ -2110,23 +2110,23 @@
         </is>
       </c>
       <c r="B7" s="15" t="n">
-        <v>8.970000000000001</v>
+        <v>8.989000000000001</v>
       </c>
       <c r="C7" s="15" t="n">
-        <v>4.991</v>
+        <v>4.945</v>
       </c>
       <c r="D7" s="15" t="inlineStr"/>
       <c r="E7" s="15" t="n">
-        <v>0.909</v>
+        <v>0.906</v>
       </c>
       <c r="F7" s="15" t="n">
-        <v>0.014</v>
+        <v>0.003</v>
       </c>
       <c r="G7" s="15" t="n">
-        <v>-0.003</v>
+        <v>-0.02</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-0.017</v>
+        <v>-0.016</v>
       </c>
       <c r="I7" s="15" t="n">
         <v>1</v>
@@ -2151,26 +2151,26 @@
         </is>
       </c>
       <c r="B8" s="15" t="n">
-        <v>3.737</v>
+        <v>3.766</v>
       </c>
       <c r="C8" s="15" t="n">
-        <v>2.285</v>
+        <v>2.268</v>
       </c>
       <c r="D8" s="15" t="inlineStr"/>
       <c r="E8" s="15" t="n">
-        <v>0.352</v>
+        <v>0.345</v>
       </c>
       <c r="F8" s="15" t="n">
-        <v>0.016</v>
+        <v>0.021</v>
       </c>
       <c r="G8" s="15" t="n">
         <v>-0.059</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>0.025</v>
+        <v>0.016</v>
       </c>
       <c r="I8" s="15" t="n">
-        <v>0.341</v>
+        <v>0.336</v>
       </c>
       <c r="J8" s="15" t="n">
         <v>1</v>
@@ -2194,29 +2194,29 @@
         </is>
       </c>
       <c r="B9" s="15" t="n">
-        <v>3.247</v>
+        <v>3.271</v>
       </c>
       <c r="C9" s="15" t="n">
-        <v>1.081</v>
+        <v>1.074</v>
       </c>
       <c r="D9" s="15" t="inlineStr"/>
       <c r="E9" s="15" t="n">
-        <v>-0.008</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="F9" s="15" t="n">
-        <v>0.095</v>
+        <v>0.104</v>
       </c>
       <c r="G9" s="15" t="n">
+        <v>-0.057</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>-0.07099999999999999</v>
+      </c>
+      <c r="I9" s="15" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="J9" s="15" t="n">
         <v>-0.043</v>
-      </c>
-      <c r="H9" s="15" t="n">
-        <v>-0.05</v>
-      </c>
-      <c r="I9" s="15" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="J9" s="15" t="n">
-        <v>-0.026</v>
       </c>
       <c r="K9" s="15" t="n">
         <v>1</v>
@@ -2239,34 +2239,34 @@
         </is>
       </c>
       <c r="B10" s="15" t="n">
-        <v>4</v>
+        <v>4.062</v>
       </c>
       <c r="C10" s="15" t="n">
-        <v>0.612</v>
+        <v>0.62</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>0.91</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>0.012</v>
+        <v>0.022</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>0.029</v>
+        <v>0.031</v>
       </c>
       <c r="G10" s="15" t="n">
-        <v>0.047</v>
+        <v>0.06</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.083</v>
       </c>
       <c r="I10" s="15" t="n">
-        <v>-0.025</v>
+        <v>-0.028</v>
       </c>
       <c r="J10" s="15" t="n">
-        <v>0.036</v>
+        <v>0.021</v>
       </c>
       <c r="K10" s="15" t="n">
-        <v>-0.011</v>
+        <v>0.05</v>
       </c>
       <c r="L10" s="15" t="n">
         <v>1</v>
@@ -2288,37 +2288,37 @@
         </is>
       </c>
       <c r="B11" s="15" t="n">
-        <v>5.023</v>
+        <v>5.046</v>
       </c>
       <c r="C11" s="15" t="n">
-        <v>0.577</v>
+        <v>0.573</v>
       </c>
       <c r="D11" s="15" t="n">
         <v>0.93</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>-0.024</v>
+        <v>-0.058</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>-0.02</v>
+        <v>-0.035</v>
       </c>
       <c r="G11" s="15" t="n">
-        <v>0.05</v>
+        <v>0.065</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>-0.079</v>
+        <v>-0.089</v>
       </c>
       <c r="I11" s="15" t="n">
-        <v>0.026</v>
+        <v>-0.014</v>
       </c>
       <c r="J11" s="15" t="n">
-        <v>-0.08</v>
+        <v>-0.083</v>
       </c>
       <c r="K11" s="15" t="n">
-        <v>-0.046</v>
+        <v>-0.051</v>
       </c>
       <c r="L11" s="15" t="n">
-        <v>-0.119</v>
+        <v>-0.149</v>
       </c>
       <c r="M11" s="15" t="n">
         <v>1</v>
@@ -2339,40 +2339,40 @@
         </is>
       </c>
       <c r="B12" s="15" t="n">
-        <v>3.467</v>
+        <v>3.469</v>
       </c>
       <c r="C12" s="15" t="n">
-        <v>0.899</v>
+        <v>0.918</v>
       </c>
       <c r="D12" s="15" t="n">
         <v>0.86</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>-0.016</v>
+        <v>-0.007</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.047</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>-0.028</v>
+        <v>-0.036</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>0.057</v>
+        <v>0.054</v>
       </c>
       <c r="I12" s="15" t="n">
-        <v>0.037</v>
+        <v>0.061</v>
       </c>
       <c r="J12" s="15" t="n">
-        <v>0.081</v>
+        <v>0.08</v>
       </c>
       <c r="K12" s="15" t="n">
-        <v>-0.039</v>
+        <v>-0.076</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>0.055</v>
+        <v>0.023</v>
       </c>
       <c r="M12" s="15" t="n">
-        <v>0.042</v>
+        <v>0.04</v>
       </c>
       <c r="N12" s="15" t="n">
         <v>1</v>
@@ -2392,43 +2392,43 @@
         </is>
       </c>
       <c r="B13" s="15" t="n">
-        <v>4.562</v>
+        <v>4.601</v>
       </c>
       <c r="C13" s="15" t="n">
-        <v>0.902</v>
+        <v>0.893</v>
       </c>
       <c r="D13" s="15" t="n">
         <v>0.84</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>-0.079</v>
+        <v>-0.077</v>
       </c>
       <c r="F13" s="15" t="n">
-        <v>-0.118</v>
+        <v>-0.077</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>-0.049</v>
+        <v>-0.073</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>0.055</v>
       </c>
       <c r="I13" s="15" t="n">
-        <v>-0.045</v>
+        <v>-0.054</v>
       </c>
       <c r="J13" s="15" t="n">
-        <v>-0.07199999999999999</v>
+        <v>-0.083</v>
       </c>
       <c r="K13" s="15" t="n">
-        <v>-0.089</v>
+        <v>-0.059</v>
       </c>
       <c r="L13" s="15" t="n">
-        <v>-0.03</v>
+        <v>-0.05</v>
       </c>
       <c r="M13" s="15" t="n">
-        <v>-0.049</v>
+        <v>-0.093</v>
       </c>
       <c r="N13" s="15" t="n">
-        <v>0.018</v>
+        <v>0.004</v>
       </c>
       <c r="O13" s="15" t="n">
         <v>1</v>
@@ -2447,46 +2447,46 @@
         </is>
       </c>
       <c r="B14" s="15" t="n">
-        <v>4.526</v>
+        <v>4.515</v>
       </c>
       <c r="C14" s="15" t="n">
-        <v>1.178</v>
+        <v>1.195</v>
       </c>
       <c r="D14" s="15" t="n">
         <v>0.88</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>-0.017</v>
+        <v>-0.001</v>
       </c>
       <c r="F14" s="15" t="n">
-        <v>-0.016</v>
+        <v>-0.029</v>
       </c>
       <c r="G14" s="15" t="n">
-        <v>-0.035</v>
+        <v>-0.043</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>0.024</v>
+        <v>0.04</v>
       </c>
       <c r="I14" s="15" t="n">
-        <v>0.045</v>
+        <v>0.056</v>
       </c>
       <c r="J14" s="15" t="n">
-        <v>-0.1</v>
+        <v>-0.064</v>
       </c>
       <c r="K14" s="15" t="n">
-        <v>-0.041</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="L14" s="15" t="n">
         <v>-0.34</v>
       </c>
       <c r="M14" s="15" t="n">
-        <v>0.33</v>
+        <v>0.357</v>
       </c>
       <c r="N14" s="15" t="n">
-        <v>-0.022</v>
+        <v>-0.013</v>
       </c>
       <c r="O14" s="15" t="n">
-        <v>-0.045</v>
+        <v>-0.044</v>
       </c>
       <c r="P14" s="15" t="n">
         <v>1</v>
@@ -2504,49 +2504,49 @@
         </is>
       </c>
       <c r="B15" s="15" t="n">
-        <v>2.956</v>
+        <v>2.996</v>
       </c>
       <c r="C15" s="15" t="n">
-        <v>1.111</v>
+        <v>1.138</v>
       </c>
       <c r="D15" s="15" t="n">
         <v>0.87</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>-0.012</v>
+        <v>-0.008</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>-0.013</v>
+        <v>0.006</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>0.006</v>
+        <v>-0.014</v>
       </c>
       <c r="H15" s="15" t="n">
         <v>-0.044</v>
       </c>
       <c r="I15" s="15" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.063</v>
       </c>
       <c r="J15" s="15" t="n">
-        <v>0.058</v>
+        <v>0.037</v>
       </c>
       <c r="K15" s="15" t="n">
-        <v>0.059</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="L15" s="15" t="n">
-        <v>0.299</v>
+        <v>0.312</v>
       </c>
       <c r="M15" s="15" t="n">
-        <v>-0.268</v>
+        <v>-0.262</v>
       </c>
       <c r="N15" s="15" t="n">
-        <v>0.028</v>
+        <v>0.022</v>
       </c>
       <c r="O15" s="15" t="n">
-        <v>-0.117</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="P15" s="15" t="n">
-        <v>-0.45</v>
+        <v>-0.446</v>
       </c>
       <c r="Q15" s="15" t="n">
         <v>1</v>
@@ -2563,52 +2563,52 @@
         </is>
       </c>
       <c r="B16" s="15" t="n">
-        <v>4.587</v>
+        <v>4.591</v>
       </c>
       <c r="C16" s="15" t="n">
-        <v>0.459</v>
+        <v>0.47</v>
       </c>
       <c r="D16" s="15" t="n">
         <v>0.9</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>-0.039</v>
+        <v>-0.025</v>
       </c>
       <c r="F16" s="15" t="n">
+        <v>-0.014</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>-0.057</v>
+      </c>
+      <c r="H16" s="15" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="I16" s="15" t="n">
+        <v>-0.038</v>
+      </c>
+      <c r="J16" s="15" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="G16" s="15" t="n">
-        <v>-0.111</v>
-      </c>
-      <c r="H16" s="15" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="I16" s="15" t="n">
-        <v>-0.044</v>
-      </c>
-      <c r="J16" s="15" t="n">
-        <v>0.002</v>
-      </c>
       <c r="K16" s="15" t="n">
-        <v>-0.016</v>
+        <v>-0.045</v>
       </c>
       <c r="L16" s="15" t="n">
-        <v>0.031</v>
+        <v>0.041</v>
       </c>
       <c r="M16" s="15" t="n">
-        <v>-0.004</v>
+        <v>0.036</v>
       </c>
       <c r="N16" s="15" t="n">
-        <v>-0.129</v>
+        <v>-0.148</v>
       </c>
       <c r="O16" s="15" t="n">
-        <v>0.014</v>
+        <v>0.038</v>
       </c>
       <c r="P16" s="15" t="n">
         <v>0.06900000000000001</v>
       </c>
       <c r="Q16" s="15" t="n">
-        <v>-0.083</v>
+        <v>-0.037</v>
       </c>
       <c r="R16" s="15" t="n">
         <v>1</v>
@@ -2624,55 +2624,55 @@
         </is>
       </c>
       <c r="B17" s="15" t="n">
-        <v>4.742</v>
+        <v>4.766</v>
       </c>
       <c r="C17" s="15" t="n">
-        <v>1.019</v>
+        <v>1.016</v>
       </c>
       <c r="D17" s="15" t="n">
         <v>0.9</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>-0.036</v>
+        <v>-0.047</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>0</v>
+        <v>-0.024</v>
       </c>
       <c r="G17" s="15" t="n">
-        <v>0.019</v>
+        <v>-0.062</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>0.026</v>
+        <v>0.039</v>
       </c>
       <c r="I17" s="15" t="n">
-        <v>-0.001</v>
+        <v>0.015</v>
       </c>
       <c r="J17" s="15" t="n">
-        <v>-0.041</v>
+        <v>-0.033</v>
       </c>
       <c r="K17" s="15" t="n">
-        <v>-0.052</v>
+        <v>-0.099</v>
       </c>
       <c r="L17" s="15" t="n">
-        <v>-0.204</v>
+        <v>-0.325</v>
       </c>
       <c r="M17" s="15" t="n">
-        <v>0.233</v>
+        <v>0.311</v>
       </c>
       <c r="N17" s="15" t="n">
-        <v>-0.007</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="O17" s="15" t="n">
-        <v>0.026</v>
+        <v>0.059</v>
       </c>
       <c r="P17" s="15" t="n">
-        <v>0.675</v>
+        <v>0.711</v>
       </c>
       <c r="Q17" s="15" t="n">
-        <v>-0.653</v>
+        <v>-0.66</v>
       </c>
       <c r="R17" s="15" t="n">
-        <v>0.064</v>
+        <v>0.035</v>
       </c>
       <c r="S17" s="15" t="n">
         <v>1</v>
@@ -2687,58 +2687,58 @@
         </is>
       </c>
       <c r="B18" s="15" t="n">
-        <v>4.625</v>
+        <v>4.859</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>1.152</v>
+        <v>1.346</v>
       </c>
       <c r="D18" s="15" t="n">
         <v>0.92</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>-0.013</v>
+        <v>-0.077</v>
       </c>
       <c r="F18" s="15" t="n">
-        <v>-0.04</v>
+        <v>-0.003</v>
       </c>
       <c r="G18" s="15" t="n">
-        <v>-0.028</v>
+        <v>-0.094</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-0.025</v>
+        <v>-0.029</v>
       </c>
       <c r="I18" s="15" t="n">
-        <v>0.011</v>
+        <v>-0.056</v>
       </c>
       <c r="J18" s="15" t="n">
-        <v>-0.008</v>
+        <v>-0.03</v>
       </c>
       <c r="K18" s="15" t="n">
-        <v>0.008999999999999999</v>
+        <v>-0.032</v>
       </c>
       <c r="L18" s="15" t="n">
-        <v>-0.401</v>
+        <v>-0.435</v>
       </c>
       <c r="M18" s="15" t="n">
-        <v>0.367</v>
+        <v>0.52</v>
       </c>
       <c r="N18" s="15" t="n">
-        <v>-0.056</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="O18" s="15" t="n">
-        <v>0.02</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="P18" s="15" t="n">
-        <v>0.353</v>
+        <v>0.427</v>
       </c>
       <c r="Q18" s="15" t="n">
-        <v>-0.343</v>
+        <v>-0.375</v>
       </c>
       <c r="R18" s="15" t="n">
-        <v>0.082</v>
+        <v>0.095</v>
       </c>
       <c r="S18" s="15" t="n">
-        <v>0.268</v>
+        <v>0.405</v>
       </c>
       <c r="T18" s="15" t="n">
         <v>1</v>
@@ -2752,61 +2752,61 @@
         </is>
       </c>
       <c r="B19" s="15" t="n">
-        <v>2.596</v>
+        <v>2.386</v>
       </c>
       <c r="C19" s="15" t="n">
-        <v>1.057</v>
+        <v>1.024</v>
       </c>
       <c r="D19" s="15" t="n">
         <v>0.89</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>0.024</v>
+        <v>-0.056</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.092</v>
       </c>
       <c r="G19" s="15" t="n">
-        <v>0.082</v>
+        <v>0.034</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-0.012</v>
+        <v>0</v>
       </c>
       <c r="I19" s="15" t="n">
-        <v>-0.02</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="J19" s="15" t="n">
-        <v>0.008999999999999999</v>
+        <v>-0.056</v>
       </c>
       <c r="K19" s="15" t="n">
-        <v>-0.007</v>
+        <v>-0.005</v>
       </c>
       <c r="L19" s="15" t="n">
-        <v>0.455</v>
+        <v>0.504</v>
       </c>
       <c r="M19" s="15" t="n">
-        <v>-0.43</v>
+        <v>-0.436</v>
       </c>
       <c r="N19" s="15" t="n">
-        <v>0.054</v>
+        <v>-0.013</v>
       </c>
       <c r="O19" s="15" t="n">
-        <v>-0.065</v>
+        <v>0.021</v>
       </c>
       <c r="P19" s="15" t="n">
-        <v>-0.43</v>
+        <v>-0.381</v>
       </c>
       <c r="Q19" s="15" t="n">
-        <v>0.35</v>
+        <v>0.325</v>
       </c>
       <c r="R19" s="15" t="n">
-        <v>-0.031</v>
+        <v>0.001</v>
       </c>
       <c r="S19" s="15" t="n">
-        <v>-0.302</v>
+        <v>-0.348</v>
       </c>
       <c r="T19" s="15" t="n">
-        <v>-0.416</v>
+        <v>-0.592</v>
       </c>
       <c r="U19" s="15" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
delivery v4.0: filled new richer 6-template structure (Model1 9 sheets, Model2 4 sheets, Model3 6 sheets, appendix 5 sheets, ICC + YUYU)
</commit_message>
<xml_diff>
--- a/results/主模型结果填答表.xlsx
+++ b/results/主模型结果填答表.xlsx
@@ -1978,10 +1978,10 @@
         </is>
       </c>
       <c r="B3" s="15" t="n">
-        <v>29.641</v>
+        <v>29.756</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>4.691</v>
+        <v>4.813</v>
       </c>
       <c r="D3" s="15" t="inlineStr"/>
       <c r="E3" s="15" t="n">
@@ -2011,14 +2011,14 @@
         </is>
       </c>
       <c r="B4" s="15" t="n">
-        <v>0.605</v>
+        <v>0.581</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>0.49</v>
+        <v>0.494</v>
       </c>
       <c r="D4" s="15" t="inlineStr"/>
       <c r="E4" s="15" t="n">
-        <v>-0.026</v>
+        <v>-0.015</v>
       </c>
       <c r="F4" s="15" t="n">
         <v>1</v>
@@ -2046,17 +2046,17 @@
         </is>
       </c>
       <c r="B5" s="15" t="n">
-        <v>3.154</v>
+        <v>3.176</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>0.895</v>
+        <v>0.888</v>
       </c>
       <c r="D5" s="15" t="inlineStr"/>
       <c r="E5" s="15" t="n">
-        <v>0.027</v>
+        <v>0.026</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>0.023</v>
+        <v>0.065</v>
       </c>
       <c r="G5" s="15" t="n">
         <v>1</v>
@@ -2083,20 +2083,20 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>2.509</v>
+        <v>2.482</v>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1.075</v>
+        <v>1.085</v>
       </c>
       <c r="D6" s="15" t="inlineStr"/>
       <c r="E6" s="15" t="n">
-        <v>-0.028</v>
+        <v>-0.037</v>
       </c>
       <c r="F6" s="15" t="n">
-        <v>0.039</v>
+        <v>0.041</v>
       </c>
       <c r="G6" s="15" t="n">
-        <v>-0.066</v>
+        <v>-0.043</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>1</v>
@@ -2122,23 +2122,23 @@
         </is>
       </c>
       <c r="B7" s="15" t="n">
-        <v>7.655</v>
+        <v>7.806</v>
       </c>
       <c r="C7" s="15" t="n">
-        <v>4.879</v>
+        <v>4.922</v>
       </c>
       <c r="D7" s="15" t="inlineStr"/>
       <c r="E7" s="15" t="n">
-        <v>0.923</v>
+        <v>0.922</v>
       </c>
       <c r="F7" s="15" t="n">
-        <v>-0.039</v>
+        <v>-0.045</v>
       </c>
       <c r="G7" s="15" t="n">
-        <v>-0.007</v>
+        <v>0.013</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-0.058</v>
+        <v>-0.062</v>
       </c>
       <c r="I7" s="15" t="n">
         <v>1</v>
@@ -2163,26 +2163,26 @@
         </is>
       </c>
       <c r="B8" s="15" t="n">
-        <v>3.497</v>
+        <v>3.579</v>
       </c>
       <c r="C8" s="15" t="n">
-        <v>2.334</v>
+        <v>2.429</v>
       </c>
       <c r="D8" s="15" t="inlineStr"/>
       <c r="E8" s="15" t="n">
-        <v>0.423</v>
+        <v>0.384</v>
       </c>
       <c r="F8" s="15" t="n">
-        <v>-0.017</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="G8" s="15" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.083</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>0.015</v>
+        <v>0.066</v>
       </c>
       <c r="I8" s="15" t="n">
-        <v>0.447</v>
+        <v>0.418</v>
       </c>
       <c r="J8" s="15" t="n">
         <v>1</v>
@@ -2206,29 +2206,29 @@
         </is>
       </c>
       <c r="B9" s="15" t="n">
-        <v>3.223</v>
+        <v>3.222</v>
       </c>
       <c r="C9" s="15" t="n">
-        <v>1.098</v>
+        <v>1.133</v>
       </c>
       <c r="D9" s="15" t="inlineStr"/>
       <c r="E9" s="15" t="n">
-        <v>0.061</v>
+        <v>0.066</v>
       </c>
       <c r="F9" s="15" t="n">
-        <v>-0.03</v>
+        <v>-0.025</v>
       </c>
       <c r="G9" s="15" t="n">
-        <v>-0.016</v>
+        <v>-0.06</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>0.073</v>
+        <v>0.089</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>0.066</v>
+        <v>0.074</v>
       </c>
       <c r="J9" s="15" t="n">
-        <v>0.082</v>
+        <v>0.124</v>
       </c>
       <c r="K9" s="15" t="n">
         <v>1</v>
@@ -2251,34 +2251,34 @@
         </is>
       </c>
       <c r="B10" s="15" t="n">
-        <v>4.03</v>
+        <v>4.045</v>
       </c>
       <c r="C10" s="15" t="n">
-        <v>0.622</v>
+        <v>0.613</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>0.91</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>0.061</v>
+        <v>0.039</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>0.039</v>
+        <v>0.036</v>
       </c>
       <c r="G10" s="15" t="n">
-        <v>0.108</v>
+        <v>0.107</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-0.032</v>
+        <v>-0.061</v>
       </c>
       <c r="I10" s="15" t="n">
-        <v>0.073</v>
+        <v>0.06</v>
       </c>
       <c r="J10" s="15" t="n">
-        <v>-0.011</v>
+        <v>-0.042</v>
       </c>
       <c r="K10" s="15" t="n">
-        <v>-0.079</v>
+        <v>-0.047</v>
       </c>
       <c r="L10" s="15" t="n">
         <v>1</v>
@@ -2300,37 +2300,37 @@
         </is>
       </c>
       <c r="B11" s="15" t="n">
-        <v>5.043</v>
+        <v>5.006</v>
       </c>
       <c r="C11" s="15" t="n">
-        <v>0.599</v>
+        <v>0.585</v>
       </c>
       <c r="D11" s="15" t="n">
         <v>0.93</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.091</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>0.083</v>
+        <v>0.059</v>
       </c>
       <c r="G11" s="15" t="n">
-        <v>0.055</v>
+        <v>0.068</v>
       </c>
       <c r="H11" s="15" t="n">
         <v>-0.078</v>
       </c>
       <c r="I11" s="15" t="n">
-        <v>-0.062</v>
+        <v>-0.08</v>
       </c>
       <c r="J11" s="15" t="n">
-        <v>0.012</v>
+        <v>0.023</v>
       </c>
       <c r="K11" s="15" t="n">
-        <v>0.006</v>
+        <v>-0.019</v>
       </c>
       <c r="L11" s="15" t="n">
-        <v>-0.165</v>
+        <v>-0.147</v>
       </c>
       <c r="M11" s="15" t="n">
         <v>1</v>
@@ -2351,40 +2351,40 @@
         </is>
       </c>
       <c r="B12" s="15" t="n">
-        <v>3.47</v>
+        <v>3.444</v>
       </c>
       <c r="C12" s="15" t="n">
-        <v>0.915</v>
+        <v>0.905</v>
       </c>
       <c r="D12" s="15" t="n">
         <v>0.86</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.005</v>
+        <v>0.031</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>0.023</v>
+        <v>0.018</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>0.018</v>
+        <v>0.044</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>0.015</v>
+        <v>0.004</v>
       </c>
       <c r="I12" s="15" t="n">
-        <v>0.054</v>
+        <v>0.076</v>
       </c>
       <c r="J12" s="15" t="n">
-        <v>-0.018</v>
+        <v>-0.012</v>
       </c>
       <c r="K12" s="15" t="n">
-        <v>0.049</v>
+        <v>0.011</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>0.042</v>
+        <v>0.025</v>
       </c>
       <c r="M12" s="15" t="n">
-        <v>0.059</v>
+        <v>0.02</v>
       </c>
       <c r="N12" s="15" t="n">
         <v>1</v>
@@ -2404,43 +2404,43 @@
         </is>
       </c>
       <c r="B13" s="15" t="n">
-        <v>4.568</v>
+        <v>4.56</v>
       </c>
       <c r="C13" s="15" t="n">
-        <v>0.898</v>
+        <v>0.884</v>
       </c>
       <c r="D13" s="15" t="n">
         <v>0.84</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>-0.021</v>
+        <v>-0.046</v>
       </c>
       <c r="F13" s="15" t="n">
-        <v>-0.04</v>
+        <v>-0.016</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>0.033</v>
+        <v>0.042</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.053</v>
       </c>
       <c r="I13" s="15" t="n">
-        <v>-0.02</v>
+        <v>-0.046</v>
       </c>
       <c r="J13" s="15" t="n">
-        <v>-0.102</v>
+        <v>-0.074</v>
       </c>
       <c r="K13" s="15" t="n">
-        <v>-0.002</v>
+        <v>0.008</v>
       </c>
       <c r="L13" s="15" t="n">
-        <v>0.053</v>
+        <v>-0.011</v>
       </c>
       <c r="M13" s="15" t="n">
-        <v>-0.062</v>
+        <v>-0.05</v>
       </c>
       <c r="N13" s="15" t="n">
-        <v>-0.018</v>
+        <v>-0.007</v>
       </c>
       <c r="O13" s="15" t="n">
         <v>1</v>
@@ -2459,46 +2459,46 @@
         </is>
       </c>
       <c r="B14" s="15" t="n">
-        <v>4.545</v>
+        <v>4.493</v>
       </c>
       <c r="C14" s="15" t="n">
-        <v>1.156</v>
+        <v>1.118</v>
       </c>
       <c r="D14" s="15" t="n">
         <v>0.88</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>-0.036</v>
+        <v>-0.012</v>
       </c>
       <c r="F14" s="15" t="n">
-        <v>-0.003</v>
+        <v>0.044</v>
       </c>
       <c r="G14" s="15" t="n">
-        <v>-0.066</v>
+        <v>-0.096</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>0.021</v>
+        <v>0.011</v>
       </c>
       <c r="I14" s="15" t="n">
-        <v>-0.044</v>
+        <v>-0.021</v>
       </c>
       <c r="J14" s="15" t="n">
-        <v>0.008</v>
+        <v>0.045</v>
       </c>
       <c r="K14" s="15" t="n">
-        <v>-0.021</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="L14" s="15" t="n">
         <v>-0.282</v>
       </c>
       <c r="M14" s="15" t="n">
-        <v>0.268</v>
+        <v>0.323</v>
       </c>
       <c r="N14" s="15" t="n">
-        <v>0.028</v>
+        <v>0.052</v>
       </c>
       <c r="O14" s="15" t="n">
-        <v>0.023</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="P14" s="15" t="n">
         <v>1</v>
@@ -2516,49 +2516,49 @@
         </is>
       </c>
       <c r="B15" s="15" t="n">
-        <v>2.86</v>
+        <v>2.898</v>
       </c>
       <c r="C15" s="15" t="n">
-        <v>1.088</v>
+        <v>1.091</v>
       </c>
       <c r="D15" s="15" t="n">
         <v>0.87</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>-0.047</v>
+        <v>-0.03</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>0.057</v>
+        <v>0.065</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>0.011</v>
+        <v>0.031</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>0.011</v>
+        <v>-0.036</v>
       </c>
       <c r="I15" s="15" t="n">
-        <v>-0.029</v>
+        <v>-0.012</v>
       </c>
       <c r="J15" s="15" t="n">
-        <v>0.068</v>
+        <v>0.015</v>
       </c>
       <c r="K15" s="15" t="n">
-        <v>-0.062</v>
+        <v>-0.022</v>
       </c>
       <c r="L15" s="15" t="n">
-        <v>0.288</v>
+        <v>0.255</v>
       </c>
       <c r="M15" s="15" t="n">
-        <v>-0.242</v>
+        <v>-0.253</v>
       </c>
       <c r="N15" s="15" t="n">
-        <v>-0.02</v>
+        <v>-0.028</v>
       </c>
       <c r="O15" s="15" t="n">
-        <v>-0.039</v>
+        <v>-0.08</v>
       </c>
       <c r="P15" s="15" t="n">
-        <v>-0.344</v>
+        <v>-0.381</v>
       </c>
       <c r="Q15" s="15" t="n">
         <v>1</v>
@@ -2575,52 +2575,52 @@
         </is>
       </c>
       <c r="B16" s="15" t="n">
-        <v>4.663</v>
+        <v>4.671</v>
       </c>
       <c r="C16" s="15" t="n">
-        <v>0.503</v>
+        <v>0.493</v>
       </c>
       <c r="D16" s="15" t="n">
         <v>0.9</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>0.05</v>
+        <v>0.061</v>
       </c>
       <c r="F16" s="15" t="n">
-        <v>0.122</v>
+        <v>0.105</v>
       </c>
       <c r="G16" s="15" t="n">
-        <v>-0.012</v>
+        <v>-0.031</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-0.041</v>
+        <v>-0.019</v>
       </c>
       <c r="I16" s="15" t="n">
-        <v>0.029</v>
+        <v>0.03</v>
       </c>
       <c r="J16" s="15" t="n">
-        <v>0.133</v>
+        <v>0.142</v>
       </c>
       <c r="K16" s="15" t="n">
-        <v>-0.04</v>
+        <v>-0.033</v>
       </c>
       <c r="L16" s="15" t="n">
-        <v>0.025</v>
+        <v>0.06</v>
       </c>
       <c r="M16" s="15" t="n">
-        <v>0.041</v>
+        <v>-0.015</v>
       </c>
       <c r="N16" s="15" t="n">
-        <v>-0.147</v>
+        <v>-0.136</v>
       </c>
       <c r="O16" s="15" t="n">
-        <v>0.016</v>
+        <v>0.044</v>
       </c>
       <c r="P16" s="15" t="n">
-        <v>-0.015</v>
+        <v>-0.032</v>
       </c>
       <c r="Q16" s="15" t="n">
-        <v>0.057</v>
+        <v>0.051</v>
       </c>
       <c r="R16" s="15" t="n">
         <v>1</v>
@@ -2636,55 +2636,55 @@
         </is>
       </c>
       <c r="B17" s="15" t="n">
-        <v>4.714</v>
+        <v>4.701</v>
       </c>
       <c r="C17" s="15" t="n">
-        <v>0.91</v>
+        <v>0.97</v>
       </c>
       <c r="D17" s="15" t="n">
         <v>0.9</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>0.058</v>
+        <v>0.04</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>-0.031</v>
+        <v>-0.01</v>
       </c>
       <c r="G17" s="15" t="n">
-        <v>-0.003</v>
+        <v>0.023</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>-0.057</v>
+        <v>0.03</v>
       </c>
       <c r="I17" s="15" t="n">
-        <v>0.019</v>
+        <v>0.008</v>
       </c>
       <c r="J17" s="15" t="n">
-        <v>-0.006</v>
+        <v>0.05</v>
       </c>
       <c r="K17" s="15" t="n">
+        <v>-0.012</v>
+      </c>
+      <c r="L17" s="15" t="n">
+        <v>-0.256</v>
+      </c>
+      <c r="M17" s="15" t="n">
+        <v>0.326</v>
+      </c>
+      <c r="N17" s="15" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="O17" s="15" t="n">
         <v>0.036</v>
       </c>
-      <c r="L17" s="15" t="n">
-        <v>-0.279</v>
-      </c>
-      <c r="M17" s="15" t="n">
-        <v>0.319</v>
-      </c>
-      <c r="N17" s="15" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="O17" s="15" t="n">
-        <v>0.062</v>
-      </c>
       <c r="P17" s="15" t="n">
-        <v>0.591</v>
+        <v>0.678</v>
       </c>
       <c r="Q17" s="15" t="n">
-        <v>-0.659</v>
+        <v>-0.643</v>
       </c>
       <c r="R17" s="15" t="n">
-        <v>-0.003</v>
+        <v>-0.077</v>
       </c>
       <c r="S17" s="15" t="n">
         <v>1</v>
@@ -2699,58 +2699,58 @@
         </is>
       </c>
       <c r="B18" s="15" t="n">
-        <v>4.805</v>
+        <v>4.758</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>1.259</v>
+        <v>1.17</v>
       </c>
       <c r="D18" s="15" t="n">
         <v>0.92</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>-0.099</v>
+        <v>-0.122</v>
       </c>
       <c r="F18" s="15" t="n">
-        <v>0.014</v>
+        <v>0.081</v>
       </c>
       <c r="G18" s="15" t="n">
-        <v>0.015</v>
+        <v>-0.074</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>0.001</v>
+        <v>0.036</v>
       </c>
       <c r="I18" s="15" t="n">
-        <v>-0.077</v>
+        <v>-0.096</v>
       </c>
       <c r="J18" s="15" t="n">
-        <v>-0.062</v>
+        <v>0.033</v>
       </c>
       <c r="K18" s="15" t="n">
-        <v>-0.051</v>
+        <v>-0.074</v>
       </c>
       <c r="L18" s="15" t="n">
-        <v>-0.459</v>
+        <v>-0.365</v>
       </c>
       <c r="M18" s="15" t="n">
-        <v>0.339</v>
+        <v>0.43</v>
       </c>
       <c r="N18" s="15" t="n">
-        <v>-0.047</v>
+        <v>0.004</v>
       </c>
       <c r="O18" s="15" t="n">
-        <v>0.057</v>
+        <v>0.019</v>
       </c>
       <c r="P18" s="15" t="n">
-        <v>0.433</v>
+        <v>0.398</v>
       </c>
       <c r="Q18" s="15" t="n">
-        <v>-0.299</v>
+        <v>-0.341</v>
       </c>
       <c r="R18" s="15" t="n">
-        <v>0.018</v>
+        <v>-0.022</v>
       </c>
       <c r="S18" s="15" t="n">
-        <v>0.338</v>
+        <v>0.332</v>
       </c>
       <c r="T18" s="15" t="n">
         <v>1</v>
@@ -2764,61 +2764,61 @@
         </is>
       </c>
       <c r="B19" s="15" t="n">
-        <v>2.511</v>
+        <v>2.381</v>
       </c>
       <c r="C19" s="15" t="n">
-        <v>1.062</v>
+        <v>1.007</v>
       </c>
       <c r="D19" s="15" t="n">
         <v>0.89</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>0.01</v>
+        <v>0.105</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>-0.057</v>
+        <v>-0.017</v>
       </c>
       <c r="G19" s="15" t="n">
-        <v>0.054</v>
+        <v>-0.053</v>
       </c>
       <c r="H19" s="15" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="I19" s="15" t="n">
         <v>0.08</v>
       </c>
-      <c r="I19" s="15" t="n">
-        <v>0.01</v>
-      </c>
       <c r="J19" s="15" t="n">
-        <v>-0.018</v>
+        <v>-0.032</v>
       </c>
       <c r="K19" s="15" t="n">
-        <v>-0.059</v>
+        <v>0.068</v>
       </c>
       <c r="L19" s="15" t="n">
-        <v>0.343</v>
+        <v>0.317</v>
       </c>
       <c r="M19" s="15" t="n">
-        <v>-0.357</v>
+        <v>-0.336</v>
       </c>
       <c r="N19" s="15" t="n">
-        <v>-0.017</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="O19" s="15" t="n">
-        <v>-0.011</v>
+        <v>0.019</v>
       </c>
       <c r="P19" s="15" t="n">
-        <v>-0.251</v>
+        <v>-0.286</v>
       </c>
       <c r="Q19" s="15" t="n">
-        <v>0.401</v>
+        <v>0.356</v>
       </c>
       <c r="R19" s="15" t="n">
-        <v>-0.064</v>
+        <v>-0.008</v>
       </c>
       <c r="S19" s="15" t="n">
-        <v>-0.352</v>
+        <v>-0.241</v>
       </c>
       <c r="T19" s="15" t="n">
-        <v>-0.289</v>
+        <v>-0.398</v>
       </c>
       <c r="U19" s="15" t="n">
         <v>1</v>

</xml_diff>